<commit_message>
test(stage): record production page and file regressions
</commit_message>
<xml_diff>
--- a/docs/stage-20260908/D/evidence/cnv-analysis-synthetic-cnv_CNV_实验记录.xlsx
+++ b/docs/stage-20260908/D/evidence/cnv-analysis-synthetic-cnv_CNV_实验记录.xlsx
@@ -498,7 +498,7 @@
         <v>待填写</v>
       </c>
       <c r="J2" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="3">
@@ -530,7 +530,7 @@
         <v>待填写</v>
       </c>
       <c r="J3" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="4">
@@ -562,7 +562,7 @@
         <v>待填写</v>
       </c>
       <c r="J4" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="5">
@@ -594,7 +594,7 @@
         <v>待填写</v>
       </c>
       <c r="J5" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="6">
@@ -626,7 +626,7 @@
         <v>待填写</v>
       </c>
       <c r="J6" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="7">
@@ -658,7 +658,7 @@
         <v>待填写</v>
       </c>
       <c r="J7" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
   </sheetData>
@@ -751,7 +751,7 @@
         <v>Generated at</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-09-08T05:50:11.009Z</v>
+        <v>2026-09-08T06:08:43.673Z</v>
       </c>
     </row>
     <row r="4">
@@ -823,7 +823,7 @@
         <v>Run / Plate / Analysis</v>
       </c>
       <c r="B12" t="str">
-        <v>synthetic-cnv / 待填写 / CNV-synthetic-cnv-20260908055010</v>
+        <v>synthetic-cnv / 待填写 / CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
   </sheetData>
@@ -870,7 +870,7 @@
         <v>Run ID / Plate ID / Analysis ID</v>
       </c>
       <c r="B3" t="str">
-        <v>synthetic-cnv / 待填写 / CNV-synthetic-cnv-20260908055010</v>
+        <v>synthetic-cnv / 待填写 / CNV-synthetic-cnv-20260908060843</v>
       </c>
       <c r="C3" t="str">
         <v>自动 + 人工</v>
@@ -1123,7 +1123,7 @@
         <v>待填写</v>
       </c>
       <c r="H2" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="3">
@@ -1149,7 +1149,7 @@
         <v>待填写</v>
       </c>
       <c r="H3" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="4">
@@ -1175,7 +1175,7 @@
         <v>待填写</v>
       </c>
       <c r="H4" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="5">
@@ -1201,7 +1201,7 @@
         <v>待填写</v>
       </c>
       <c r="H5" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="6">
@@ -1227,7 +1227,7 @@
         <v>待填写</v>
       </c>
       <c r="H6" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
   </sheetData>
@@ -1400,7 +1400,7 @@
         <v>待填写</v>
       </c>
       <c r="W2" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="3">
@@ -1465,7 +1465,7 @@
         <v>待填写</v>
       </c>
       <c r="W3" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="4">
@@ -1530,7 +1530,7 @@
         <v>待填写</v>
       </c>
       <c r="W4" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="5">
@@ -1595,7 +1595,7 @@
         <v>待填写</v>
       </c>
       <c r="W5" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="6">
@@ -1660,7 +1660,7 @@
         <v>待填写</v>
       </c>
       <c r="W6" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="7">
@@ -1725,7 +1725,7 @@
         <v>待填写</v>
       </c>
       <c r="W7" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
   </sheetData>
@@ -1911,7 +1911,7 @@
         <v>待填写</v>
       </c>
       <c r="X2" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="3">
@@ -1985,7 +1985,7 @@
         <v>待填写</v>
       </c>
       <c r="X3" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="4">
@@ -2059,7 +2059,7 @@
         <v>待填写</v>
       </c>
       <c r="X4" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="5">
@@ -2133,7 +2133,7 @@
         <v>待填写</v>
       </c>
       <c r="X5" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="6">
@@ -2207,7 +2207,7 @@
         <v>待填写</v>
       </c>
       <c r="X6" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="7">
@@ -2281,7 +2281,7 @@
         <v>待填写</v>
       </c>
       <c r="X7" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
   </sheetData>
@@ -2526,7 +2526,7 @@
         <v>待填写</v>
       </c>
       <c r="AL2" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="3">
@@ -2603,7 +2603,7 @@
         <v>待填写</v>
       </c>
       <c r="AL3" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="4">
@@ -2680,7 +2680,7 @@
         <v>待填写</v>
       </c>
       <c r="AL4" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="5">
@@ -2757,7 +2757,7 @@
         <v>待填写</v>
       </c>
       <c r="AL5" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="6">
@@ -2834,7 +2834,7 @@
         <v>待填写</v>
       </c>
       <c r="AL6" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="7">
@@ -2911,7 +2911,7 @@
         <v>待填写</v>
       </c>
       <c r="AL7" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="8">
@@ -2988,7 +2988,7 @@
         <v>待填写</v>
       </c>
       <c r="AL8" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="9">
@@ -3065,7 +3065,7 @@
         <v>待填写</v>
       </c>
       <c r="AL9" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="10">
@@ -3142,7 +3142,7 @@
         <v>待填写</v>
       </c>
       <c r="AL10" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="11">
@@ -3219,7 +3219,7 @@
         <v>待填写</v>
       </c>
       <c r="AL11" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="12">
@@ -3296,7 +3296,7 @@
         <v>待填写</v>
       </c>
       <c r="AL12" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="13">
@@ -3373,7 +3373,7 @@
         <v>待填写</v>
       </c>
       <c r="AL13" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="14">
@@ -3450,7 +3450,7 @@
         <v>待填写</v>
       </c>
       <c r="AL14" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="15">
@@ -3527,7 +3527,7 @@
         <v>待填写</v>
       </c>
       <c r="AL15" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="16">
@@ -3604,7 +3604,7 @@
         <v>待填写</v>
       </c>
       <c r="AL16" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="17">
@@ -3681,7 +3681,7 @@
         <v>待填写</v>
       </c>
       <c r="AL17" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="18">
@@ -3758,7 +3758,7 @@
         <v>待填写</v>
       </c>
       <c r="AL18" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="19">
@@ -3835,7 +3835,7 @@
         <v>待填写</v>
       </c>
       <c r="AL19" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="20">
@@ -3912,7 +3912,7 @@
         <v>待填写</v>
       </c>
       <c r="AL20" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="21">
@@ -3989,7 +3989,7 @@
         <v>待填写</v>
       </c>
       <c r="AL21" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="22">
@@ -4066,7 +4066,7 @@
         <v>待填写</v>
       </c>
       <c r="AL22" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="23">
@@ -4143,7 +4143,7 @@
         <v>待填写</v>
       </c>
       <c r="AL23" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="24">
@@ -4220,7 +4220,7 @@
         <v>待填写</v>
       </c>
       <c r="AL24" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="25">
@@ -4297,7 +4297,7 @@
         <v>待填写</v>
       </c>
       <c r="AL25" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="26">
@@ -4374,7 +4374,7 @@
         <v>待填写</v>
       </c>
       <c r="AL26" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="27">
@@ -4451,7 +4451,7 @@
         <v>待填写</v>
       </c>
       <c r="AL27" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="28">
@@ -4528,7 +4528,7 @@
         <v>待填写</v>
       </c>
       <c r="AL28" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="29">
@@ -4605,7 +4605,7 @@
         <v>待填写</v>
       </c>
       <c r="AL29" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="30">
@@ -4682,7 +4682,7 @@
         <v>待填写</v>
       </c>
       <c r="AL30" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="31">
@@ -4759,7 +4759,7 @@
         <v>待填写</v>
       </c>
       <c r="AL31" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="32">
@@ -4836,7 +4836,7 @@
         <v>待填写</v>
       </c>
       <c r="AL32" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="33">
@@ -4913,7 +4913,7 @@
         <v>待填写</v>
       </c>
       <c r="AL33" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="34">
@@ -4990,7 +4990,7 @@
         <v>待填写</v>
       </c>
       <c r="AL34" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="35">
@@ -5067,7 +5067,7 @@
         <v>待填写</v>
       </c>
       <c r="AL35" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="36">
@@ -5144,7 +5144,7 @@
         <v>待填写</v>
       </c>
       <c r="AL36" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="37">
@@ -5221,7 +5221,7 @@
         <v>待填写</v>
       </c>
       <c r="AL37" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="38">
@@ -5298,7 +5298,7 @@
         <v>待填写</v>
       </c>
       <c r="AL38" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="39">
@@ -5375,7 +5375,7 @@
         <v>待填写</v>
       </c>
       <c r="AL39" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="40">
@@ -5452,7 +5452,7 @@
         <v>待填写</v>
       </c>
       <c r="AL40" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="41">
@@ -5529,7 +5529,7 @@
         <v>待填写</v>
       </c>
       <c r="AL41" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="42">
@@ -5606,7 +5606,7 @@
         <v>待填写</v>
       </c>
       <c r="AL42" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="43">
@@ -5683,7 +5683,7 @@
         <v>待填写</v>
       </c>
       <c r="AL43" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="44">
@@ -5760,7 +5760,7 @@
         <v>待填写</v>
       </c>
       <c r="AL44" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="45">
@@ -5837,7 +5837,7 @@
         <v>待填写</v>
       </c>
       <c r="AL45" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="46">
@@ -5914,7 +5914,7 @@
         <v>待填写</v>
       </c>
       <c r="AL46" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="47">
@@ -5991,7 +5991,7 @@
         <v>待填写</v>
       </c>
       <c r="AL47" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="48">
@@ -6068,7 +6068,7 @@
         <v>待填写</v>
       </c>
       <c r="AL48" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="49">
@@ -6145,7 +6145,7 @@
         <v>待填写</v>
       </c>
       <c r="AL49" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
   </sheetData>
@@ -6437,7 +6437,7 @@
         <v>待填写</v>
       </c>
       <c r="T2" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
   </sheetData>
@@ -6490,7 +6490,7 @@
         <v>待填写</v>
       </c>
       <c r="E2" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="3">
@@ -6507,7 +6507,7 @@
         <v>待填写</v>
       </c>
       <c r="E3" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="4">
@@ -6524,7 +6524,7 @@
         <v>待填写</v>
       </c>
       <c r="E4" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="5">
@@ -6541,7 +6541,7 @@
         <v>待填写</v>
       </c>
       <c r="E5" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="6">
@@ -6558,7 +6558,7 @@
         <v>待填写</v>
       </c>
       <c r="E6" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="7">
@@ -6575,7 +6575,7 @@
         <v>待填写</v>
       </c>
       <c r="E7" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="8">
@@ -6592,7 +6592,7 @@
         <v>待填写</v>
       </c>
       <c r="E8" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="9">
@@ -6609,7 +6609,7 @@
         <v>待填写</v>
       </c>
       <c r="E9" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="10">
@@ -6626,7 +6626,7 @@
         <v>待填写</v>
       </c>
       <c r="E10" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="11">
@@ -6643,7 +6643,7 @@
         <v>待填写</v>
       </c>
       <c r="E11" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="12">
@@ -6660,7 +6660,7 @@
         <v>待填写</v>
       </c>
       <c r="E12" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="13">
@@ -6677,7 +6677,7 @@
         <v>待填写</v>
       </c>
       <c r="E13" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="14">
@@ -6694,7 +6694,7 @@
         <v>待填写</v>
       </c>
       <c r="E14" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="15">
@@ -6711,7 +6711,7 @@
         <v>待填写</v>
       </c>
       <c r="E15" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="16">
@@ -6728,7 +6728,7 @@
         <v>待填写</v>
       </c>
       <c r="E16" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
     <row r="17">
@@ -6745,7 +6745,7 @@
         <v>待填写</v>
       </c>
       <c r="E17" t="str">
-        <v>CNV-synthetic-cnv-20260908055010</v>
+        <v>CNV-synthetic-cnv-20260908060843</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(stage): publish unified acceptance and reproducible evidence
</commit_message>
<xml_diff>
--- a/docs/stage-20260908/D/evidence/cnv-analysis-synthetic-cnv_CNV_实验记录.xlsx
+++ b/docs/stage-20260908/D/evidence/cnv-analysis-synthetic-cnv_CNV_实验记录.xlsx
@@ -498,7 +498,7 @@
         <v>待填写</v>
       </c>
       <c r="J2" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="3">
@@ -530,7 +530,7 @@
         <v>待填写</v>
       </c>
       <c r="J3" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="4">
@@ -562,7 +562,7 @@
         <v>待填写</v>
       </c>
       <c r="J4" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="5">
@@ -594,7 +594,7 @@
         <v>待填写</v>
       </c>
       <c r="J5" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="6">
@@ -626,7 +626,7 @@
         <v>待填写</v>
       </c>
       <c r="J6" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="7">
@@ -658,7 +658,7 @@
         <v>待填写</v>
       </c>
       <c r="J7" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
   </sheetData>
@@ -751,7 +751,7 @@
         <v>Generated at</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-09-08T06:08:43.673Z</v>
+        <v>2026-09-08T06:17:23.244Z</v>
       </c>
     </row>
     <row r="4">
@@ -823,7 +823,7 @@
         <v>Run / Plate / Analysis</v>
       </c>
       <c r="B12" t="str">
-        <v>synthetic-cnv / 待填写 / CNV-synthetic-cnv-20260908060843</v>
+        <v>synthetic-cnv / 待填写 / CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
   </sheetData>
@@ -870,7 +870,7 @@
         <v>Run ID / Plate ID / Analysis ID</v>
       </c>
       <c r="B3" t="str">
-        <v>synthetic-cnv / 待填写 / CNV-synthetic-cnv-20260908060843</v>
+        <v>synthetic-cnv / 待填写 / CNV-synthetic-cnv-20260908061723</v>
       </c>
       <c r="C3" t="str">
         <v>自动 + 人工</v>
@@ -1123,7 +1123,7 @@
         <v>待填写</v>
       </c>
       <c r="H2" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="3">
@@ -1149,7 +1149,7 @@
         <v>待填写</v>
       </c>
       <c r="H3" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="4">
@@ -1175,7 +1175,7 @@
         <v>待填写</v>
       </c>
       <c r="H4" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="5">
@@ -1201,7 +1201,7 @@
         <v>待填写</v>
       </c>
       <c r="H5" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="6">
@@ -1227,7 +1227,7 @@
         <v>待填写</v>
       </c>
       <c r="H6" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
   </sheetData>
@@ -1400,7 +1400,7 @@
         <v>待填写</v>
       </c>
       <c r="W2" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="3">
@@ -1465,7 +1465,7 @@
         <v>待填写</v>
       </c>
       <c r="W3" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="4">
@@ -1530,7 +1530,7 @@
         <v>待填写</v>
       </c>
       <c r="W4" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="5">
@@ -1595,7 +1595,7 @@
         <v>待填写</v>
       </c>
       <c r="W5" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="6">
@@ -1660,7 +1660,7 @@
         <v>待填写</v>
       </c>
       <c r="W6" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="7">
@@ -1725,7 +1725,7 @@
         <v>待填写</v>
       </c>
       <c r="W7" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
   </sheetData>
@@ -1911,7 +1911,7 @@
         <v>待填写</v>
       </c>
       <c r="X2" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="3">
@@ -1985,7 +1985,7 @@
         <v>待填写</v>
       </c>
       <c r="X3" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="4">
@@ -2059,7 +2059,7 @@
         <v>待填写</v>
       </c>
       <c r="X4" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="5">
@@ -2133,7 +2133,7 @@
         <v>待填写</v>
       </c>
       <c r="X5" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="6">
@@ -2207,7 +2207,7 @@
         <v>待填写</v>
       </c>
       <c r="X6" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="7">
@@ -2281,7 +2281,7 @@
         <v>待填写</v>
       </c>
       <c r="X7" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
   </sheetData>
@@ -2526,7 +2526,7 @@
         <v>待填写</v>
       </c>
       <c r="AL2" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="3">
@@ -2603,7 +2603,7 @@
         <v>待填写</v>
       </c>
       <c r="AL3" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="4">
@@ -2680,7 +2680,7 @@
         <v>待填写</v>
       </c>
       <c r="AL4" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="5">
@@ -2757,7 +2757,7 @@
         <v>待填写</v>
       </c>
       <c r="AL5" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="6">
@@ -2834,7 +2834,7 @@
         <v>待填写</v>
       </c>
       <c r="AL6" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="7">
@@ -2911,7 +2911,7 @@
         <v>待填写</v>
       </c>
       <c r="AL7" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="8">
@@ -2988,7 +2988,7 @@
         <v>待填写</v>
       </c>
       <c r="AL8" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="9">
@@ -3065,7 +3065,7 @@
         <v>待填写</v>
       </c>
       <c r="AL9" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="10">
@@ -3142,7 +3142,7 @@
         <v>待填写</v>
       </c>
       <c r="AL10" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="11">
@@ -3219,7 +3219,7 @@
         <v>待填写</v>
       </c>
       <c r="AL11" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="12">
@@ -3296,7 +3296,7 @@
         <v>待填写</v>
       </c>
       <c r="AL12" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="13">
@@ -3373,7 +3373,7 @@
         <v>待填写</v>
       </c>
       <c r="AL13" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="14">
@@ -3450,7 +3450,7 @@
         <v>待填写</v>
       </c>
       <c r="AL14" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="15">
@@ -3527,7 +3527,7 @@
         <v>待填写</v>
       </c>
       <c r="AL15" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="16">
@@ -3604,7 +3604,7 @@
         <v>待填写</v>
       </c>
       <c r="AL16" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="17">
@@ -3681,7 +3681,7 @@
         <v>待填写</v>
       </c>
       <c r="AL17" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="18">
@@ -3758,7 +3758,7 @@
         <v>待填写</v>
       </c>
       <c r="AL18" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="19">
@@ -3835,7 +3835,7 @@
         <v>待填写</v>
       </c>
       <c r="AL19" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="20">
@@ -3912,7 +3912,7 @@
         <v>待填写</v>
       </c>
       <c r="AL20" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="21">
@@ -3989,7 +3989,7 @@
         <v>待填写</v>
       </c>
       <c r="AL21" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="22">
@@ -4066,7 +4066,7 @@
         <v>待填写</v>
       </c>
       <c r="AL22" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="23">
@@ -4143,7 +4143,7 @@
         <v>待填写</v>
       </c>
       <c r="AL23" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="24">
@@ -4220,7 +4220,7 @@
         <v>待填写</v>
       </c>
       <c r="AL24" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="25">
@@ -4297,7 +4297,7 @@
         <v>待填写</v>
       </c>
       <c r="AL25" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="26">
@@ -4374,7 +4374,7 @@
         <v>待填写</v>
       </c>
       <c r="AL26" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="27">
@@ -4451,7 +4451,7 @@
         <v>待填写</v>
       </c>
       <c r="AL27" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="28">
@@ -4528,7 +4528,7 @@
         <v>待填写</v>
       </c>
       <c r="AL28" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="29">
@@ -4605,7 +4605,7 @@
         <v>待填写</v>
       </c>
       <c r="AL29" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="30">
@@ -4682,7 +4682,7 @@
         <v>待填写</v>
       </c>
       <c r="AL30" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="31">
@@ -4759,7 +4759,7 @@
         <v>待填写</v>
       </c>
       <c r="AL31" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="32">
@@ -4836,7 +4836,7 @@
         <v>待填写</v>
       </c>
       <c r="AL32" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="33">
@@ -4913,7 +4913,7 @@
         <v>待填写</v>
       </c>
       <c r="AL33" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="34">
@@ -4990,7 +4990,7 @@
         <v>待填写</v>
       </c>
       <c r="AL34" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="35">
@@ -5067,7 +5067,7 @@
         <v>待填写</v>
       </c>
       <c r="AL35" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="36">
@@ -5144,7 +5144,7 @@
         <v>待填写</v>
       </c>
       <c r="AL36" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="37">
@@ -5221,7 +5221,7 @@
         <v>待填写</v>
       </c>
       <c r="AL37" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="38">
@@ -5298,7 +5298,7 @@
         <v>待填写</v>
       </c>
       <c r="AL38" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="39">
@@ -5375,7 +5375,7 @@
         <v>待填写</v>
       </c>
       <c r="AL39" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="40">
@@ -5452,7 +5452,7 @@
         <v>待填写</v>
       </c>
       <c r="AL40" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="41">
@@ -5529,7 +5529,7 @@
         <v>待填写</v>
       </c>
       <c r="AL41" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="42">
@@ -5606,7 +5606,7 @@
         <v>待填写</v>
       </c>
       <c r="AL42" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="43">
@@ -5683,7 +5683,7 @@
         <v>待填写</v>
       </c>
       <c r="AL43" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="44">
@@ -5760,7 +5760,7 @@
         <v>待填写</v>
       </c>
       <c r="AL44" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="45">
@@ -5837,7 +5837,7 @@
         <v>待填写</v>
       </c>
       <c r="AL45" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="46">
@@ -5914,7 +5914,7 @@
         <v>待填写</v>
       </c>
       <c r="AL46" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="47">
@@ -5991,7 +5991,7 @@
         <v>待填写</v>
       </c>
       <c r="AL47" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="48">
@@ -6068,7 +6068,7 @@
         <v>待填写</v>
       </c>
       <c r="AL48" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="49">
@@ -6145,7 +6145,7 @@
         <v>待填写</v>
       </c>
       <c r="AL49" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
   </sheetData>
@@ -6437,7 +6437,7 @@
         <v>待填写</v>
       </c>
       <c r="T2" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
   </sheetData>
@@ -6490,7 +6490,7 @@
         <v>待填写</v>
       </c>
       <c r="E2" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="3">
@@ -6507,7 +6507,7 @@
         <v>待填写</v>
       </c>
       <c r="E3" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="4">
@@ -6524,7 +6524,7 @@
         <v>待填写</v>
       </c>
       <c r="E4" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="5">
@@ -6541,7 +6541,7 @@
         <v>待填写</v>
       </c>
       <c r="E5" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="6">
@@ -6558,7 +6558,7 @@
         <v>待填写</v>
       </c>
       <c r="E6" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="7">
@@ -6575,7 +6575,7 @@
         <v>待填写</v>
       </c>
       <c r="E7" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="8">
@@ -6592,7 +6592,7 @@
         <v>待填写</v>
       </c>
       <c r="E8" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="9">
@@ -6609,7 +6609,7 @@
         <v>待填写</v>
       </c>
       <c r="E9" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="10">
@@ -6626,7 +6626,7 @@
         <v>待填写</v>
       </c>
       <c r="E10" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="11">
@@ -6643,7 +6643,7 @@
         <v>待填写</v>
       </c>
       <c r="E11" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="12">
@@ -6660,7 +6660,7 @@
         <v>待填写</v>
       </c>
       <c r="E12" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="13">
@@ -6677,7 +6677,7 @@
         <v>待填写</v>
       </c>
       <c r="E13" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="14">
@@ -6694,7 +6694,7 @@
         <v>待填写</v>
       </c>
       <c r="E14" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="15">
@@ -6711,7 +6711,7 @@
         <v>待填写</v>
       </c>
       <c r="E15" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="16">
@@ -6728,7 +6728,7 @@
         <v>待填写</v>
       </c>
       <c r="E16" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
     <row r="17">
@@ -6745,7 +6745,7 @@
         <v>待填写</v>
       </c>
       <c r="E17" t="str">
-        <v>CNV-synthetic-cnv-20260908060843</v>
+        <v>CNV-synthetic-cnv-20260908061723</v>
       </c>
     </row>
   </sheetData>

</xml_diff>